<commit_message>
sch+BOM: re-source C4/C13/C27 off the order-only 10uF 0603 to a stocked part
GRM188R61A106KE69D (10uF 10V X5R 0603) is Active but DigiKey stocks/prices no
variation (order-only), so all three bulk caps were unpriced. Re-sourced to
GRM188R61A106ME69D -- same 10uF/10V/X5R/0603, tolerance K->M (+-10%->+-20%,
immaterial for bulk/decoupling on the STO, VDD, and LED-anode nodes) -- DK
490-10475-1-ND, Active, $0.12 @1, 578k in stock. MPN updated in both the
schematic (all 3 instances: C4/C13/C27) and the master xlsx; package unchanged
(0603), so nets and copper are untouched. A 25V drop-in (GRM188R61E106MA73D,
$0.26) is noted in the row for extra DC-bias margin if wanted.

Subtotal -> $134.90 / 48 priced cells; the only ordered line still unpriced is
U8/AEM10300 (Mouser-pending).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015D4iTho3BuNxSQyJmyaxvg
</commit_message>
<xml_diff>
--- a/PCB/solar-glow-drh-v4_0-BOM.xlsx
+++ b/PCB/solar-glow-drh-v4_0-BOM.xlsx
@@ -1315,11 +1315,15 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>GRM188R61A106KE69D</t>
-        </is>
-      </c>
-      <c r="H15" s="14" t="n"/>
-      <c r="I15" s="14" t="n"/>
+          <t>GRM188R61A106ME69D</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>0.12</v>
+      </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
           <t>LAND REWORK</t>
@@ -1327,7 +1331,7 @@
       </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>Bumped 4.7uF 0402 -&gt; 10uF 10V 0603 for more effective VS bulk (stiffer rail under glow / NFC-inrush / accel transients). 0603 land - PCB rework. DK live-verified 2026-07-22: 490-10474-1-ND, Active, but DK API returned no qty-1 standard price (non-stock/order item); ~$0.15 class - confirm at cart.</t>
+          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)</t>
         </is>
       </c>
       <c r="L15" s="11" t="inlineStr">
@@ -1337,7 +1341,7 @@
       </c>
       <c r="M15" s="11" t="inlineStr">
         <is>
-          <t>490-10474-1-ND</t>
+          <t>490-10475-1-ND</t>
         </is>
       </c>
     </row>
@@ -2287,11 +2291,15 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>GRM188R61A106KE69D</t>
-        </is>
-      </c>
-      <c r="H31" s="14" t="n"/>
-      <c r="I31" s="14" t="n"/>
+          <t>GRM188R61A106ME69D</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I31" s="14" t="n">
+        <v>0.12</v>
+      </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
           <t>LAND REWORK</t>
@@ -2299,13 +2307,13 @@
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
-          <t>Bumped 4.7uF 0402 -&gt; 10uF 10V 0603; keeps the glow-PWM transient off the shared VS rail. 0603 land - PCB rework. DK live-verified 2026-07-22: 490-10474-1-ND, Active, but DK API returned no qty-1 standard price (non-stock/order item); ~$0.15 class - confirm at cart.</t>
+          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)</t>
         </is>
       </c>
       <c r="L31" s="11" t="n"/>
       <c r="M31" s="11" t="inlineStr">
         <is>
-          <t>490-10474-1-ND</t>
+          <t>490-10475-1-ND</t>
         </is>
       </c>
     </row>
@@ -2810,10 +2818,10 @@
           <t>GRM155R61E105MA12D</t>
         </is>
       </c>
-      <c r="H40" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I40" t="n">
+      <c r="H40" s="8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I40" s="8" t="n">
         <v>0.1</v>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -3087,8 +3095,14 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>GRM188R61A106KE69D</t>
-        </is>
+          <t>GRM188R61A106ME69D</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.12</v>
       </c>
       <c r="J45" s="8" t="inlineStr">
         <is>
@@ -3097,12 +3111,12 @@
       </c>
       <c r="K45" s="8" t="inlineStr">
         <is>
-          <t>Moved to 0603 to keep 10uF at 10V (per request; matches C25's approach). STO rides to 4.65V where a 6.3V 0402 was thin + heavily derated; 10V 0603 gives full margin and effective bulk. Shares the C4/C13 10uF 10V 0603 reel. Land grows from 0402 - PCB rework. DK live-verified 2026-07-22: 490-10474-1-ND, Active, but DK API returned no qty-1 standard price (non-stock/order item); ~$0.15 class - confirm at cart.</t>
+          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)</t>
         </is>
       </c>
       <c r="M45" s="8" t="inlineStr">
         <is>
-          <t>490-10474-1-ND</t>
+          <t>490-10475-1-ND</t>
         </is>
       </c>
     </row>
@@ -3640,11 +3654,11 @@
         </is>
       </c>
       <c r="I56" s="8" t="n">
-        <v>134.54</v>
+        <v>134.9</v>
       </c>
       <c r="K56" s="8" t="inlineStr">
         <is>
-          <t>Sum of the 45 priced Ext$ cells only - a few lines remain unpriced (C4/C13/C27 10uF 0603 no DK price; U8/AEM10300 Mouser-pending). See footnote.</t>
+          <t>Sum of the 48 priced Ext$ cells only - the only remaining unpriced ordered line is U8/AEM10300 (Mouser-pending). See footnote.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BOM: longevity/stability parts pass, rebuilt on the uploaded board files
Re-applies the GRM->GRT / RC->AC / precision-divider / AEC-Q100-U6 pass (see
prior PR #58 description) on top of the 2026-07-23 SCH/PCB upload, which was
exported before that pass and would otherwise have reverted it. The upload's
Supplier P/N fields (PR #57) were retained by the export and stay intact; the
BOM xlsx and TODO carry over unchanged from the original pass.

Same content as before: 31 refs re-MPN'd (ceramics to GRT AEC-Q200 with V/tol
bumps, resistors to AC AEC-Q200, R5/R6 to RE0402BRE071ML 0.1%/50ppm, U6 to
TPS22918TDBVRQ1), 4 descriptions corrected, supplier P/Ns refreshed.
Cross-check schematic<->BOM MPNs: clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015D4iTho3BuNxSQyJmyaxvg
</commit_message>
<xml_diff>
--- a/PCB/solar-glow-drh-v4_0-BOM.xlsx
+++ b/PCB/solar-glow-drh-v4_0-BOM.xlsx
@@ -827,7 +827,7 @@
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>RC0402FR-07150RL</t>
+          <t>AC0402FR-07150RL</t>
         </is>
       </c>
       <c r="H7" s="14" t="n">
@@ -843,7 +843,7 @@
       </c>
       <c r="K7" s="13" t="inlineStr">
         <is>
-          <t>Package corrected to 0402 to match the placed land (BOM previously listed 1206; a 1206 part will not fit). 1/16 W is ample (~12 mW peak/LED). Value still SIZED for the clamped ~3.47 V rail (~9 mA/LED peak); re-tune after the energy-budget bench test. Any 0402 150 Ω 1% equivalent works (esp. for PCBA sourcing). DK live-verified 2026-07-22: 311-150LRCT-ND, Active, $0.10 @1 (DKPN corrected from format-derived guess).</t>
+          <t>Package corrected to 0402 to match the placed land (BOM previously listed 1206; a 1206 part will not fit). 1/16 W is ample (~12 mW peak/LED). Value still SIZED for the clamped ~3.47 V rail (~9 mA/LED peak); re-tune after the energy-budget bench test. Any 0402 150 Ω 1% equivalent works (esp. for PCBA sourcing). DK live-verified 2026-07-22: 311-150LRCT-ND, Active, $0.10 @1 (DKPN corrected from format-derived guess).  UPGRADED 2026-07-23 (longevity): Yageo RC-&gt;AC (AEC-Q200 automotive grade), same value/tol. DK YAG3443CT-ND, $0.1 @1, Active.</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="M7" s="11" t="inlineStr">
         <is>
-          <t>311-150LRCT-ND</t>
+          <t>YAG3443CT-ND</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>RC0402FR-07220RL</t>
+          <t>AC0402FR-07220RL</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
@@ -904,7 +904,7 @@
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>Sets the SW2 TINY dim level; tunable. [v3.0: 0402 to match board land; price TBC] DK live-verified 2026-07-22: 311-220LRCT-ND, Active, $0.10 @1 (DKPN corrected).</t>
+          <t>Sets the SW2 TINY dim level; tunable. [v3.0: 0402 to match board land; price TBC] DK live-verified 2026-07-22: 311-220LRCT-ND, Active, $0.10 @1 (DKPN corrected).  UPGRADED 2026-07-23 (longevity): Yageo RC-&gt;AC (AEC-Q200 automotive grade), same value/tol. DK YAG3456CT-ND, $0.1 @1, Active.</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="M8" s="11" t="inlineStr">
         <is>
-          <t>311-220LRCT-ND</t>
+          <t>YAG3456CT-ND</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>1 MΩ, ±1%</t>
+          <t>1 MΩ, ±0.1%</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -949,14 +949,14 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>RC0402FR-071ML</t>
+          <t>RE0402BRE071ML</t>
         </is>
       </c>
       <c r="H9" s="14" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
@@ -965,7 +965,7 @@
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>R5=R6 → VSENSE = VIN/2 (tracks light, ~0 V dark). Feeds ADC + the AC0 wake-on-light comparator. [v3.0: 0402 to match board land; price TBC] DK live-verified 2026-07-22: 311-1.00MLRCT-ND, Active, $0.10 @1 (DKPN corrected).</t>
+          <t>R5=R6 → VSENSE = VIN/2 (tracks light, ~0 V dark). Feeds ADC + the AC0 wake-on-light comparator. [v3.0: 0402 to match board land; price TBC] DK live-verified 2026-07-22: 311-1.00MLRCT-ND, Active, $0.10 @1 (DKPN corrected).  UPGRADED 2026-07-23 (stability): precision Yageo RE, 0.1% / 50 ppm (VSENSE divider ratio + drift). DK 13-RE0402BRE071MLCT-ND, $0.30 @1, Active. (True thin-film not available at 1M in 0402; RE precision thick-film is the best in-footprint option.)</t>
         </is>
       </c>
       <c r="L9" s="11" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="M9" s="11" t="inlineStr">
         <is>
-          <t>311-1.00MLRCT-ND</t>
+          <t>13-RE0402BRE071MLCT-ND</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>100 nF, X7R, 16 V</t>
+          <t>100 nF, X7R, 50 V</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H10" s="14" t="n">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>RC filter on the VSENSE node. [v3.0: 0402 to match board land; price TBC] [consolidation: 10nF -&gt; 100nF, joins the 100 nF group] DK live-verified 2026-07-22: DKPN corrected from GRM155R71C103KA01D-ND (a 10nF part, stale from the 10nF-&gt;100nF consolidation) to 490-3261-1-ND (100nF, matches the KA88D MPN). Active, $0.10 @1.</t>
+          <t>RC filter on the VSENSE node. [v3.0: 0402 to match board land; price TBC] [consolidation: 10nF -&gt; 100nF, joins the 100 nF group] DK live-verified 2026-07-22: DKPN corrected from GRM155R71C103KA01D-ND (a 10nF part, stale from the 10nF-&gt;100nF consolidation) to 490-3261-1-ND (100nF, matches the KA88D MPN). Active, $0.10 @1.  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="M10" s="11" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>RC0402FR-074K7L</t>
+          <t>AC0402FR-074K7L</t>
         </is>
       </c>
       <c r="H12" s="14" t="n">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>Required — open-drain TWI bus. Firmware must set TWIROUTEA = ALT2. [v3.0: 0402 to match board land; price TBC] DK live-verified 2026-07-22: 311-4.7KLRCT-ND, Active, $0.10 @1 (DKPN corrected).</t>
+          <t>Required — open-drain TWI bus. Firmware must set TWIROUTEA = ALT2. [v3.0: 0402 to match board land; price TBC] DK live-verified 2026-07-22: 311-4.7KLRCT-ND, Active, $0.10 @1 (DKPN corrected).  UPGRADED 2026-07-23 (longevity): Yageo RC-&gt;AC (AEC-Q200 automotive grade), same value/tol. DK YAG3497CT-ND, $0.1 @1, Active.</t>
         </is>
       </c>
       <c r="L12" s="11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="M12" s="11" t="inlineStr">
         <is>
-          <t>311-4.7KLRCT-ND</t>
+          <t>YAG3497CT-ND</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>100 nF, X7R, 16 V</t>
+          <t>100 nF, X7R, 50 V</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H13" s="14" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="K13" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [v3.0: 0402 to match board land; price TBC] DK verified 2026-07-02 via this MPN: 490-3261-1-ND, $0.10 @ 1 CT; C3/C6/C7/C8 are the same line item.</t>
+          <t xml:space="preserve"> [v3.0: 0402 to match board land; price TBC] DK verified 2026-07-02 via this MPN: 490-3261-1-ND, $0.10 @ 1 CT; C3/C6/C7/C8 are the same line item.  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="M13" s="11" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>100 nF, X7R, 16 V</t>
+          <t>100 nF, X7R, 50 V</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
@@ -1254,14 +1254,14 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H14" s="14" t="n">
         <v>0.1</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [v3.0: 0402 to match board land; price TBC]</t>
+          <t xml:space="preserve"> [v3.0: 0402 to match board land; price TBC]  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="L14" s="11" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="M14" s="11" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>10 µF, X5R, 10 V</t>
+          <t>10 µF, X5R, 16 V</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
@@ -1315,14 +1315,14 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>GRM188R61A106ME69D</t>
+          <t>GRT188R61C106KE13D</t>
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.12</v>
+        <v>0.29</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>0.12</v>
+        <v>0.29</v>
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)</t>
+          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-12317-1-ND, $0.29 @1, Active. 10-&gt;16 V, 20-&gt;10% tol.</t>
         </is>
       </c>
       <c r="L15" s="11" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="M15" s="11" t="inlineStr">
         <is>
-          <t>490-10475-1-ND</t>
+          <t>490-12317-1-ND</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>100 nF, X7R, 16 V</t>
+          <t>100 nF, X7R, 50 V</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H16" s="14" t="n">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [v3.0: 0402 to match board land; price TBC]</t>
+          <t xml:space="preserve"> [v3.0: 0402 to match board land; price TBC]  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="L16" s="11" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>GRM155R71C224KA12D</t>
+          <t>GRT155R71C224KE01D</t>
         </is>
       </c>
       <c r="H17" s="14" t="n">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>ADXL367 pin 9 VREG_OUT1 → GND. Datasheet-mandated 0.2 µF; 0.22 µF nearest std. DK live-verified 2026-07-22: 490-5418-1-ND, Active, $0.10 @1 (DKPN filled).</t>
+          <t>ADXL367 pin 9 VREG_OUT1 → GND. Datasheet-mandated 0.2 µF; 0.22 µF nearest std. DK live-verified 2026-07-22: 490-5418-1-ND, Active, $0.10 @1 (DKPN filled).  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71C224KE01DCT-ND, $0.1 @1, Active.</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="M17" s="11" t="inlineStr">
         <is>
-          <t>490-5418-1-ND</t>
+          <t>490-GRT155R71C224KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>100 nF, X7R, 16 V</t>
+          <t>100 nF, X7R, 50 V</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H18" s="14" t="n">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="K18" s="13" t="inlineStr">
         <is>
-          <t>ADXL367 pin 12 VDDIO → GND.</t>
+          <t>ADXL367 pin 12 VDDIO → GND.  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="L18" s="11" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>100 nF, X7R, 16 V</t>
+          <t>100 nF, X7R, 50 V</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -1559,14 +1559,14 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H19" s="14" t="n">
         <v>0.1</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> [v3.0: 0402 to match board land; price TBC]</t>
+          <t xml:space="preserve"> [v3.0: 0402 to match board land; price TBC]  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="L19" s="11" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="M19" s="11" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>100 nF, X7R, 16 V</t>
+          <t>100 nF, X7R, 50 V</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H29" s="14" t="n">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="K29" s="13" t="inlineStr">
         <is>
-          <t>v2.2 NFC addition. Same part as C1/C2/C3/C6/C7. [v3.0: 0402 to match board land; price TBC]</t>
+          <t>v2.2 NFC addition. Same part as C1/C2/C3/C6/C7. [v3.0: 0402 to match board land; price TBC]  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="L29" s="11" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="M29" s="11" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>10 µF, X5R, 10 V</t>
+          <t>10 µF, X5R, 16 V</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
@@ -2291,14 +2291,14 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>GRM188R61A106ME69D</t>
+          <t>GRT188R61C106KE13D</t>
         </is>
       </c>
       <c r="H31" s="14" t="n">
-        <v>0.12</v>
+        <v>0.29</v>
       </c>
       <c r="I31" s="14" t="n">
-        <v>0.12</v>
+        <v>0.29</v>
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
@@ -2307,13 +2307,13 @@
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
-          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)</t>
+          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-12317-1-ND, $0.29 @1, Active. 10-&gt;16 V, 20-&gt;10% tol.</t>
         </is>
       </c>
       <c r="L31" s="11" t="n"/>
       <c r="M31" s="11" t="inlineStr">
         <is>
-          <t>490-10475-1-ND</t>
+          <t>490-12317-1-ND</t>
         </is>
       </c>
     </row>
@@ -2409,14 +2409,14 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>TPS22918DBVR</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="H33" s="8" t="n">
-        <v>0.55</v>
+        <v>0.75</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>0.55</v>
+        <v>0.75</v>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>v3.0 addition. VIN=VS, VOUT=VNFC, ON=NFC_EN, QOD strapped to VOUT (internal RPD ~25 ohm discharge), CT floating (sanctioned per DS). Pin map VERIFIED against TI SLVSD76C (TPS22918 Rev C, repo datasheets/U6  TPS22918DBVR  $0.55.pdf; the -Q1 doc SLVSCZ8B matches identically) 2026-07-02 -- check caught a real board defect (VIN/VOUT + GND/QOD transposed on the symbol); fixed on the board same day. $0.55 @ qty 1 (DigiKey, 2026-07-02). ISD 0.5 uA typ / 3.5 uA max standing draw on VS when off. DK live-verified 2026-07-22: 296-46278-1-ND, Active, $0.55 @1 (DKPN filled).</t>
+          <t>v3.0 addition. VIN=VS, VOUT=VNFC, ON=NFC_EN, QOD strapped to VOUT (internal RPD ~25 ohm discharge), CT floating (sanctioned per DS). Pin map VERIFIED against TI SLVSD76C (TPS22918 Rev C, repo datasheets/U6  TPS22918DBVR  $0.55.pdf; the -Q1 doc SLVSCZ8B matches identically) 2026-07-02 -- check caught a real board defect (VIN/VOUT + GND/QOD transposed on the symbol); fixed on the board same day. $0.55 @ qty 1 (DigiKey, 2026-07-02). ISD 0.5 uA typ / 3.5 uA max standing draw on VS when off. DK live-verified 2026-07-22: 296-46278-1-ND, Active, $0.55 @1 (DKPN filled).  UPGRADED 2026-07-23: AEC-Q100 automotive drop-in TPS22918TDBVRQ1 (pin-identical, same die as TPS22918DBVR) -- fixes the zero-stock DBVR AND upgrades reliability. DK 296-44632-1-ND, $0.75 @1, 882 stock.</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="M33" s="8" t="inlineStr">
         <is>
-          <t>296-46278-1-ND</t>
+          <t>296-44632-1-ND</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>RC0402FR-071ML</t>
+          <t>AC0402FR-071ML</t>
         </is>
       </c>
       <c r="H34" s="8" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>v3.0 addition, placed with the R14 board patch. Consolidated 100 kΩ -&gt; 1 MΩ (joins the R5/R6/R16/R17 reel, RC0402FR-071ML). DK live-verified 2026-07-22: 311-1.00MLRCT-ND, Active, $0.10 @1 (DKPN corrected).</t>
+          <t>v3.0 addition, placed with the R14 board patch. Consolidated 100 kΩ -&gt; 1 MΩ (joins the R5/R6/R16/R17 reel, RC0402FR-071ML). DK live-verified 2026-07-22: 311-1.00MLRCT-ND, Active, $0.10 @1 (DKPN corrected).  UPGRADED 2026-07-23 (longevity): Yageo RC-&gt;AC (AEC-Q200 automotive grade), same value/tol. DK YAG3450CT-ND, $0.1 @1, Active.</t>
         </is>
       </c>
       <c r="L34" s="8" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="M34" s="8" t="inlineStr">
         <is>
-          <t>311-1.00MLRCT-ND</t>
+          <t>YAG3450CT-ND</t>
         </is>
       </c>
     </row>
@@ -2821,14 +2821,14 @@
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>GRM155R61E105MA12D</t>
+          <t>GRT155R61E105KE01J</t>
         </is>
       </c>
       <c r="H40" s="8" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="I40" s="8" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="J40" s="8" t="inlineStr">
         <is>
@@ -2837,12 +2837,12 @@
       </c>
       <c r="K40" s="8" t="inlineStr">
         <is>
-          <t>v4 LDO input cap on the STO island (~5.5 V). Original GRM155R61A105KE15D (1 uF 10 V) is obsolete and the whole Murata GRM155 1 uF 10 V 0402 X5R family is EOL. RE-SOURCED 2026-07-22 -&gt; GRM155R61E105MA12D (1 uF 25 V X5R 0402), DK 490-10018-1-ND, Active, $0.10 @1, 461k in stock. 25 V chosen for DC-bias headroom on the ~5.5 V node. Schematic MPN updated to match.</t>
+          <t>v4 LDO input cap on the STO island (~5.5 V). Original GRM155R61A105KE15D (1 uF 10 V) is obsolete and the whole Murata GRM155 1 uF 10 V 0402 X5R family is EOL. RE-SOURCED 2026-07-22 -&gt; GRM155R61E105MA12D (1 uF 25 V X5R 0402), DK 490-10018-1-ND, Active, $0.10 @1, 461k in stock. 25 V chosen for DC-bias headroom on the ~5.5 V node. Schematic MPN updated to match.  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R61E105KE01JCT-ND, $0.12 @1, Active. 20-&gt;10% tol.</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
         <is>
-          <t>490-10018-1-ND</t>
+          <t>490-GRT155R61E105KE01JCT-ND</t>
         </is>
       </c>
     </row>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>2.2 µF, 10 V, 0402, X5R</t>
+          <t>2.2 µF, 25 V, 0402, X5R</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -2877,14 +2877,14 @@
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>GRM155R61A225KE01J</t>
+          <t>GRT155R61E225KE13D</t>
         </is>
       </c>
       <c r="H41" s="8" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
@@ -2893,12 +2893,12 @@
       </c>
       <c r="K41" s="8" t="inlineStr">
         <is>
-          <t>v4 LDO output cap on VS (3.3 V). Original GRM155R61A225KE11D returned no DK results. RE-SOURCED 2026-07-22 -&gt; GRM155R61A225KE01J (2.2 uF 10 V X5R 0402, same spec), DK 490-GRM155R61A225KE01JCT-ND, Active, $0.10 @1, 38k in stock. Schematic MPN updated to match.</t>
+          <t>v4 LDO output cap on VS (3.3 V). Original GRM155R61A225KE11D returned no DK results. RE-SOURCED 2026-07-22 -&gt; GRM155R61A225KE01J (2.2 uF 10 V X5R 0402, same spec), DK 490-GRM155R61A225KE01JCT-ND, Active, $0.10 @1, 38k in stock. Schematic MPN updated to match.  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-12267-1-ND, $0.25 @1, Active. 10-&gt;25 V (LDO-loop stability).</t>
         </is>
       </c>
       <c r="M41" s="8" t="inlineStr">
         <is>
-          <t>490-GRM155R61A225KE01JCT-ND</t>
+          <t>490-12267-1-ND</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2933,7 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H42" s="8" t="n">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="K42" s="8" t="inlineStr">
         <is>
-          <t>Reuses the project 100 nF 0402 part. DK live-verified 2026-07-22: 490-3261-1-ND, Active, $0.10 @1.</t>
+          <t>Reuses the project 100 nF 0402 part. DK live-verified 2026-07-22: 490-3261-1-ND, Active, $0.10 @1.  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -2989,14 +2989,14 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>GRM188R61A226ME15D</t>
+          <t>GRT188R61A226ME13D</t>
         </is>
       </c>
       <c r="H43" s="8" t="n">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="J43" s="8" t="inlineStr">
         <is>
@@ -3005,12 +3005,12 @@
       </c>
       <c r="K43" s="8" t="inlineStr">
         <is>
-          <t>AEM10300 datasheet Table 11 CSRC = GRM188R61A226ME15D (22 uF, 10 V, X5R, 0603). 10 V rating (was 6.3 V) keeps usable capacitance at the SRC node, which rides toward panel Voc ~4.15 V where a 6.3 V X5R 0603 derates hard. DK live-verified 2026-07-22: 490-10476-1-ND, Active, $0.16 @1 (DKPN + price filled).</t>
+          <t>AEM10300 datasheet Table 11 CSRC = GRM188R61A226ME15D (22 uF, 10 V, X5R, 0603). 10 V rating (was 6.3 V) keeps usable capacitance at the SRC node, which rides toward panel Voc ~4.15 V where a 6.3 V X5R 0603 derates hard. DK live-verified 2026-07-22: 490-10476-1-ND, Active, $0.16 @1 (DKPN + price filled).  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT188R61A226ME13DCT-ND, $0.31 @1, Active. Also fixes the zero-stock GRM188R61A226ME15D.</t>
         </is>
       </c>
       <c r="M43" s="8" t="inlineStr">
         <is>
-          <t>490-10476-1-ND</t>
+          <t>490-GRT188R61A226ME13DCT-ND</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>10 uF, 0402, X5R</t>
+          <t>10 uF, 10 V, 0402, X5R</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -3045,14 +3045,14 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>GRM155R60J106ME05D</t>
+          <t>GRT155R61A106ME13J</t>
         </is>
       </c>
       <c r="H44" s="8" t="n">
-        <v>0.1</v>
+        <v>0.28</v>
       </c>
       <c r="I44" s="8" t="n">
-        <v>0.1</v>
+        <v>0.28</v>
       </c>
       <c r="J44" s="8" t="inlineStr">
         <is>
@@ -3061,12 +3061,12 @@
       </c>
       <c r="K44" s="8" t="inlineStr">
         <is>
-          <t>v4 AEM VINT buffer cap (6.3 V rail). Original GRM155R60J106ME44D discontinued at DK. RE-SOURCED 2026-07-22 -&gt; GRM155R60J106ME05D (10 uF 6.3 V X5R 0402, same spec), DK 490-GRM155R60J106ME05DCT-ND, Active, $0.10 @1, 1.2M in stock. Schematic MPN updated to match.</t>
+          <t>v4 AEM VINT buffer cap (6.3 V rail). Original GRM155R60J106ME44D discontinued at DK. RE-SOURCED 2026-07-22 -&gt; GRM155R60J106ME05D (10 uF 6.3 V X5R 0402, same spec), DK 490-GRM155R60J106ME05DCT-ND, Active, $0.10 @1, 1.2M in stock. Schematic MPN updated to match.  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R61A106ME13JCT-ND, $0.28 @1, Active. 6.3-&gt;10 V margin.</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
         <is>
-          <t>490-GRM155R60J106ME05DCT-ND</t>
+          <t>490-GRT155R61A106ME13JCT-ND</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>10 µF, 10 V, 0603, X5R</t>
+          <t>10 µF, 16 V, 0603, X5R</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -3101,14 +3101,14 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>GRM188R61A106ME69D</t>
+          <t>GRT188R61C106KE13D</t>
         </is>
       </c>
       <c r="H45" s="8" t="n">
-        <v>0.12</v>
+        <v>0.29</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>0.12</v>
+        <v>0.29</v>
       </c>
       <c r="J45" s="8" t="inlineStr">
         <is>
@@ -3117,12 +3117,12 @@
       </c>
       <c r="K45" s="8" t="inlineStr">
         <is>
-          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)</t>
+          <t>10 uF 10 V X5R 0603. Original GRM188R61A106KE69D is Active but DigiKey stocks/prices no variation (order-only). RE-SOURCED 2026-07-22 -&gt; GRM188R61A106ME69D (same 10 uF/10 V/X5R/0603, tol K-&gt;M i.e. +-10%-&gt;+-20%, immaterial for bulk/decoupling), DK 490-10475-1-ND, Active, $0.12 @1, 578k in stock. Schematic MPN updated to match. (For more DC-bias margin on the STO/LED nodes, GRM188R61E106MA73D 25 V, DK 490-7202-1-ND, $0.26 is a drop-in.)  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-12317-1-ND, $0.29 @1, Active. 10-&gt;16 V, 20-&gt;10% tol.</t>
         </is>
       </c>
       <c r="M45" s="8" t="inlineStr">
         <is>
-          <t>490-10475-1-ND</t>
+          <t>490-12317-1-ND</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>GRM155R71C104KA88D</t>
+          <t>GRT155R71H104KE01D</t>
         </is>
       </c>
       <c r="H46" s="8" t="n">
@@ -3173,12 +3173,12 @@
       </c>
       <c r="K46" s="8" t="inlineStr">
         <is>
-          <t>Reuses the project 100 nF 0402 part. DK live-verified 2026-07-22: 490-3261-1-ND, Active, $0.10 @1.</t>
+          <t>Reuses the project 100 nF 0402 part. DK live-verified 2026-07-22: 490-3261-1-ND, Active, $0.10 @1.  UPGRADED 2026-07-23 (longevity): GRM-&gt;GRT (Murata AEC-Q200 automotive grade). DK 490-GRT155R71H104KE01DCT-ND, $0.1 @1, Active. 16-&gt;50 V margin.</t>
         </is>
       </c>
       <c r="M46" s="8" t="inlineStr">
         <is>
-          <t>490-3261-1-ND</t>
+          <t>490-GRT155R71H104KE01DCT-ND</t>
         </is>
       </c>
     </row>
@@ -3213,7 +3213,7 @@
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>RC0402FR-072ML</t>
+          <t>AC0402FR-072ML</t>
         </is>
       </c>
       <c r="H47" s="8" t="n">
@@ -3229,12 +3229,12 @@
       </c>
       <c r="K47" s="8" t="inlineStr">
         <is>
-          <t>2 M in the project Yageo RC0402FR-07 1% convention; confirm at cart. DK live-verified 2026-07-22: 13-RC0402FR-072MLCT-ND, Active, $0.10 @1 (DKPN corrected).</t>
+          <t>2 M in the project Yageo RC0402FR-07 1% convention; confirm at cart. DK live-verified 2026-07-22: 13-RC0402FR-072MLCT-ND, Active, $0.10 @1 (DKPN corrected).  UPGRADED 2026-07-23 (longevity): Yageo RC-&gt;AC (AEC-Q200 automotive grade), same value/tol. DK 13-AC0402FR-072MLCT-ND, $0.1 @1, Active. No 0.1%/50ppm thin-film exists at 2M in 0402, so grade-only.</t>
         </is>
       </c>
       <c r="M47" s="8" t="inlineStr">
         <is>
-          <t>13-RC0402FR-072MLCT-ND</t>
+          <t>13-AC0402FR-072MLCT-ND</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>RC0402FR-071ML</t>
+          <t>AC0402FR-071ML</t>
         </is>
       </c>
       <c r="H48" s="8" t="n">
@@ -3285,12 +3285,12 @@
       </c>
       <c r="K48" s="8" t="inlineStr">
         <is>
-          <t>Reuses the project 1 M part (shared with R5/R6/R14). DK live-verified 2026-07-22: 311-1.00MLRCT-ND, Active, $0.10 @1 (DKPN corrected).</t>
+          <t>Reuses the project 1 M part (shared with R5/R6/R14). DK live-verified 2026-07-22: 311-1.00MLRCT-ND, Active, $0.10 @1 (DKPN corrected).  UPGRADED 2026-07-23 (longevity): Yageo RC-&gt;AC (AEC-Q200 automotive grade), same value/tol. DK YAG3450CT-ND, $0.1 @1, Active. (R16 STO-sense bottom; the R15 2M partner has no 0402 precision option, so this leg stays AEC-Q200 grade.)</t>
         </is>
       </c>
       <c r="M48" s="8" t="inlineStr">
         <is>
-          <t>311-1.00MLRCT-ND</t>
+          <t>YAG3450CT-ND</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
         </is>
       </c>
       <c r="I56" s="8" t="n">
-        <v>138.67</v>
+        <v>140.08</v>
       </c>
       <c r="K56" s="8" t="inlineStr">
         <is>
@@ -3671,7 +3671,7 @@
     <row r="58">
       <c r="A58" s="15" t="inlineStr">
         <is>
-          <t>*≈$/ea is indicative (qty 1–10, USD, ~2026) for a board-cost sanity check only — confirm live pricing at order. Supercaps + solar cells dominate. Mounting holes, SW2 and the SBn bridges carry no ordered part; the NFC coil is PCB-etched copper (no ordered part); headers (J1) unpopulated. Lineage: the old solar-glow-drh-BOM.xlsx is the v0-prototype record; v2.2 added the NFC tag (U5) + C8/C9/R13. v3.0 adds U6 (TPS22918 VNFC load switch) + R14 (100 k NFC_EN pulldown) and converts every passive except SJ1 to 0402 to match the board lands — converted/added lines have prices blanked pending a fresh quote.  |  DigiKey P/Ns and MPN status verified against live DigiKey listings 2026-07-02; per-row notes carry the evidence level (verbatim-observed vs format-derived vs page-verified).  Supercaps (SS17 3-153-440 / WS17 3-153-438) live-verified via DigiKey 2026-07-22. Full BOM re-verified live against DigiKey 2026-07-22: format-derived DK P/Ns replaced with real ones, prices refreshed, and C22/C23/C26 flagged (see rows).</t>
+          <t>*≈$/ea is indicative (qty 1–10, USD, ~2026) for a board-cost sanity check only — confirm live pricing at order. Supercaps + solar cells dominate. Mounting holes, SW2 and the SBn bridges carry no ordered part; the NFC coil is PCB-etched copper (no ordered part); headers (J1) unpopulated. Lineage: the old solar-glow-drh-BOM.xlsx is the v0-prototype record; v2.2 added the NFC tag (U5) + C8/C9/R13. v3.0 adds U6 (TPS22918 VNFC load switch) + R14 (100 k NFC_EN pulldown) and converts every passive except SJ1 to 0402 to match the board lands — converted/added lines have prices blanked pending a fresh quote.  |  DigiKey P/Ns and MPN status verified against live DigiKey listings 2026-07-02; per-row notes carry the evidence level (verbatim-observed vs format-derived vs page-verified).  Supercaps (SS17 3-153-440 / WS17 3-153-438) live-verified via DigiKey 2026-07-22. Full BOM re-verified live against DigiKey 2026-07-22: format-derived DK P/Ns replaced with real ones, prices refreshed, and C22/C23/C26 flagged (see rows).  Longevity/stability pass 2026-07-23: ceramics GRM-&gt;GRT (AEC-Q200) with V/tol bumps; resistors RC-&gt;AC (AEC-Q200), VSENSE divider R5/R6 to 0.1%/50ppm Yageo RE; U6 to AEC-Q100 TPS22918TDBVRQ1 (also clears the two zero-stock lines C25 + U6). Same footprints/values -- no layout change.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datasheets+BOM: file the missing U9 TPS7A0233 datasheet
Doc-hygiene gap from the cross-domain audit prep: U9 was the only
silicon part with no datasheet in datasheets/. Fetched TI SBVS277C
(full 48-page rev C) as 'U9  TPS7A0233PDBVR  $0.84.pdf' per the repo
naming convention and pointed the BOM row's 'Datasheet (repo)' cell
(previously empty) at it.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015D4iTho3BuNxSQyJmyaxvg
</commit_message>
<xml_diff>
--- a/PCB/solar-glow-drh-v4_0-BOM.xlsx
+++ b/PCB/solar-glow-drh-v4_0-BOM.xlsx
@@ -2611,6 +2611,11 @@
           <t>Verified active on DigiKey (product 12165099): TPS7A0233PDBVR, SOT-23-5, 200 mA nanopower LDO (TI TPS7A02 family, ~25 nA Iq). No repo datasheet. DK live-verified 2026-07-22: 296-TPS7A0233PDBVRCT-ND (DK 12165099), Active, $0.84 @1.</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>U9  TPS7A0233PDBVR  $0.84.pdf</t>
+        </is>
+      </c>
       <c r="M36" s="8" t="inlineStr">
         <is>
           <t>296-TPS7A0233PDBVRCT-ND</t>

</xml_diff>